<commit_message>
fix: #REF! errors in Grade 4 excel template
</commit_message>
<xml_diff>
--- a/public/templates/Rekord Template - Grade 4.xlsx
+++ b/public/templates/Rekord Template - Grade 4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jerwin\Documents\GitHub\rekord\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E64F626-63E4-45AF-AE22-A641E889DE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31092D7-21D8-43C9-9CE7-FAF2008C5B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README!" sheetId="5" r:id="rId1"/>
@@ -823,17 +823,8 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -843,6 +834,15 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1223,344 +1223,344 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:18" ht="87.65" customHeight="1" x14ac:dyDescent="1.2">
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="39" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
     </row>
     <row r="2" spans="3:18" ht="69.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="38"/>
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+      <c r="O2" s="38"/>
+      <c r="P2" s="38"/>
+      <c r="Q2" s="38"/>
+      <c r="R2" s="38"/>
     </row>
     <row r="3" spans="3:18" ht="22.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
-      <c r="O3" s="43"/>
-      <c r="P3" s="43"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="43"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
     </row>
     <row r="4" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="42" t="s">
         <v>123</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="39"/>
-      <c r="O4" s="39"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="42"/>
+      <c r="O4" s="42"/>
+      <c r="P4" s="42"/>
+      <c r="Q4" s="42"/>
+      <c r="R4" s="42"/>
     </row>
     <row r="5" spans="3:18" ht="40.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="41" t="s">
         <v>134</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="41"/>
+      <c r="N5" s="41"/>
+      <c r="O5" s="41"/>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="41"/>
+      <c r="R5" s="41"/>
     </row>
     <row r="6" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="38"/>
-      <c r="Q6" s="38"/>
-      <c r="R6" s="38"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="37"/>
+      <c r="M6" s="37"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
     </row>
     <row r="7" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-      <c r="R7" s="39"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="42"/>
+      <c r="O7" s="42"/>
+      <c r="P7" s="42"/>
+      <c r="Q7" s="42"/>
+      <c r="R7" s="42"/>
     </row>
     <row r="8" spans="3:18" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="37"/>
-      <c r="M8" s="37"/>
-      <c r="N8" s="37"/>
-      <c r="O8" s="37"/>
-      <c r="P8" s="37"/>
-      <c r="Q8" s="37"/>
-      <c r="R8" s="37"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="41"/>
+      <c r="I8" s="41"/>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41"/>
+      <c r="L8" s="41"/>
+      <c r="M8" s="41"/>
+      <c r="N8" s="41"/>
+      <c r="O8" s="41"/>
+      <c r="P8" s="41"/>
+      <c r="Q8" s="41"/>
+      <c r="R8" s="41"/>
     </row>
     <row r="9" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
-      <c r="O9" s="38"/>
-      <c r="P9" s="38"/>
-      <c r="Q9" s="38"/>
-      <c r="R9" s="38"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="37"/>
+      <c r="Q9" s="37"/>
+      <c r="R9" s="37"/>
     </row>
     <row r="10" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="42" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="39"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="42"/>
+      <c r="N10" s="42"/>
+      <c r="O10" s="42"/>
+      <c r="P10" s="42"/>
+      <c r="Q10" s="42"/>
+      <c r="R10" s="42"/>
     </row>
     <row r="11" spans="3:18" ht="59.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
-      <c r="L11" s="37"/>
-      <c r="M11" s="37"/>
-      <c r="N11" s="37"/>
-      <c r="O11" s="37"/>
-      <c r="P11" s="37"/>
-      <c r="Q11" s="37"/>
-      <c r="R11" s="37"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="41"/>
+      <c r="N11" s="41"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41"/>
+      <c r="Q11" s="41"/>
+      <c r="R11" s="41"/>
     </row>
     <row r="12" spans="3:18" ht="378.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="40" t="e" vm="1">
+      <c r="C12" s="43" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="40"/>
-      <c r="P12" s="40"/>
-      <c r="Q12" s="40"/>
-      <c r="R12" s="40"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="43"/>
+      <c r="L12" s="43"/>
+      <c r="M12" s="43"/>
+      <c r="N12" s="43"/>
+      <c r="O12" s="43"/>
+      <c r="P12" s="43"/>
+      <c r="Q12" s="43"/>
+      <c r="R12" s="43"/>
     </row>
     <row r="13" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="37" t="s">
         <v>132</v>
       </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="38"/>
-      <c r="K13" s="38"/>
-      <c r="L13" s="38"/>
-      <c r="M13" s="38"/>
-      <c r="N13" s="38"/>
-      <c r="O13" s="38"/>
-      <c r="P13" s="38"/>
-      <c r="Q13" s="38"/>
-      <c r="R13" s="38"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
+      <c r="F13" s="37"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="37"/>
+      <c r="I13" s="37"/>
+      <c r="J13" s="37"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="37"/>
+      <c r="M13" s="37"/>
+      <c r="N13" s="37"/>
+      <c r="O13" s="37"/>
+      <c r="P13" s="37"/>
+      <c r="Q13" s="37"/>
+      <c r="R13" s="37"/>
     </row>
     <row r="14" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39"/>
-      <c r="M14" s="39"/>
-      <c r="N14" s="39"/>
-      <c r="O14" s="39"/>
-      <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-      <c r="R14" s="39"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="42"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="42"/>
+      <c r="N14" s="42"/>
+      <c r="O14" s="42"/>
+      <c r="P14" s="42"/>
+      <c r="Q14" s="42"/>
+      <c r="R14" s="42"/>
     </row>
     <row r="15" spans="3:18" ht="41.35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
-      <c r="L15" s="37"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="37"/>
-      <c r="O15" s="37"/>
-      <c r="P15" s="37"/>
-      <c r="Q15" s="37"/>
-      <c r="R15" s="37"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="41"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="41"/>
+      <c r="L15" s="41"/>
+      <c r="M15" s="41"/>
+      <c r="N15" s="41"/>
+      <c r="O15" s="41"/>
+      <c r="P15" s="41"/>
+      <c r="Q15" s="41"/>
+      <c r="R15" s="41"/>
     </row>
     <row r="16" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="38"/>
-      <c r="N16" s="38"/>
-      <c r="O16" s="38"/>
-      <c r="P16" s="38"/>
-      <c r="Q16" s="38"/>
-      <c r="R16" s="38"/>
+      <c r="D16" s="37"/>
+      <c r="E16" s="37"/>
+      <c r="F16" s="37"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="37"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="37"/>
+      <c r="M16" s="37"/>
+      <c r="N16" s="37"/>
+      <c r="O16" s="37"/>
+      <c r="P16" s="37"/>
+      <c r="Q16" s="37"/>
+      <c r="R16" s="37"/>
     </row>
     <row r="17" spans="3:18" ht="31.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="41" t="s">
         <v>133</v>
       </c>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="37"/>
-      <c r="K17" s="37"/>
-      <c r="L17" s="37"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="37"/>
-      <c r="O17" s="37"/>
-      <c r="P17" s="37"/>
-      <c r="Q17" s="37"/>
-      <c r="R17" s="37"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="41"/>
+      <c r="K17" s="41"/>
+      <c r="L17" s="41"/>
+      <c r="M17" s="41"/>
+      <c r="N17" s="41"/>
+      <c r="O17" s="41"/>
+      <c r="P17" s="41"/>
+      <c r="Q17" s="41"/>
+      <c r="R17" s="41"/>
     </row>
     <row r="18" spans="3:18" ht="63.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="36"/>
@@ -1591,6 +1591,13 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="C2eitg/wVVV0kyyQJC0VLipqMFRM+3PW1MeezuIv/PreHWXO+QjsttCqX7YqnNPJ2EZxrPDwoJR8DE/zQIjV1w==" saltValue="4eH05uxoVOqJ721VkYCI5w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="17">
+    <mergeCell ref="C17:R17"/>
+    <mergeCell ref="C16:R16"/>
+    <mergeCell ref="C10:R10"/>
+    <mergeCell ref="C11:R11"/>
+    <mergeCell ref="C14:R14"/>
+    <mergeCell ref="C15:R15"/>
+    <mergeCell ref="C12:R12"/>
     <mergeCell ref="C6:R6"/>
     <mergeCell ref="C9:R9"/>
     <mergeCell ref="C13:R13"/>
@@ -1601,13 +1608,6 @@
     <mergeCell ref="C4:R4"/>
     <mergeCell ref="C7:R7"/>
     <mergeCell ref="C8:R8"/>
-    <mergeCell ref="C17:R17"/>
-    <mergeCell ref="C16:R16"/>
-    <mergeCell ref="C10:R10"/>
-    <mergeCell ref="C11:R11"/>
-    <mergeCell ref="C14:R14"/>
-    <mergeCell ref="C15:R15"/>
-    <mergeCell ref="C12:R12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C6:R6" location="'Class Info'!A1" display="Go to Class Info Sheet →" xr:uid="{8C8433A5-16A5-4B84-8E34-CC7C8D28B64C}"/>
@@ -42833,65 +42833,65 @@
       </c>
     </row>
     <row r="102" spans="1:74" x14ac:dyDescent="0.3">
-      <c r="A102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="B102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F102" s="9" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O102" s="6" t="e">
-        <f>IF('Class Info'!#REF!="","", 'Class Info'!#REF!)</f>
-        <v>#REF!</v>
+      <c r="A102" s="6" t="str">
+        <f>IF('Class Info'!A102="","", 'Class Info'!A102)</f>
+        <v/>
+      </c>
+      <c r="B102" s="6" t="str">
+        <f>IF('Class Info'!B102="","", 'Class Info'!B102)</f>
+        <v/>
+      </c>
+      <c r="C102" s="6" t="str">
+        <f>IF('Class Info'!C102="","", 'Class Info'!C102)</f>
+        <v/>
+      </c>
+      <c r="D102" s="6" t="str">
+        <f>IF('Class Info'!D102="","", 'Class Info'!D102)</f>
+        <v/>
+      </c>
+      <c r="E102" s="6" t="str">
+        <f>IF('Class Info'!E102="","", 'Class Info'!E102)</f>
+        <v/>
+      </c>
+      <c r="F102" s="9" t="str">
+        <f>IF('Class Info'!F102="","", 'Class Info'!F102)</f>
+        <v/>
+      </c>
+      <c r="G102" s="6" t="str">
+        <f>IF('Class Info'!G102="","", 'Class Info'!G102)</f>
+        <v/>
+      </c>
+      <c r="H102" s="6" t="str">
+        <f>IF('Class Info'!H102="","", 'Class Info'!H102)</f>
+        <v/>
+      </c>
+      <c r="I102" s="6" t="str">
+        <f>IF('Class Info'!I102="","", 'Class Info'!I102)</f>
+        <v/>
+      </c>
+      <c r="J102" s="6" t="str">
+        <f>IF('Class Info'!J102="","", 'Class Info'!J102)</f>
+        <v/>
+      </c>
+      <c r="K102" s="6" t="str">
+        <f>IF('Class Info'!K102="","", 'Class Info'!K102)</f>
+        <v/>
+      </c>
+      <c r="L102" s="6" t="str">
+        <f>IF('Class Info'!L102="","", 'Class Info'!L102)</f>
+        <v/>
+      </c>
+      <c r="M102" s="6" t="str">
+        <f>IF('Class Info'!M102="","", 'Class Info'!M102)</f>
+        <v/>
+      </c>
+      <c r="N102" s="6" t="str">
+        <f>IF('Class Info'!N102="","", 'Class Info'!N102)</f>
+        <v/>
+      </c>
+      <c r="O102" s="6" t="str">
+        <f>IF('Class Info'!O102="","", 'Class Info'!O102)</f>
+        <v/>
       </c>
       <c r="P102" s="6" t="str">
         <f>IF(Grades!D102="","", Grades!D102)</f>
@@ -43131,7 +43131,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="CzY33G6GHKcY6lkGolawmCO4F9KGgN1fQ5Jlgn9bAXezucBHq2EdMIQ3TSPcT4/CmpepbTa9hFGqrZfOLKD+Kw==" saltValue="VqXXRei/awkqPVq4Uzd10g==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="CbeBVCUfbKpoicVt+SogpIQrd9r0RB2Bjkuv/zgMXZuWFvp8NVIXs3gEvyccPQB14xu7jgG1Dfn410LpVCcTRg==" saltValue="ia4xEArnHXy/DQeCa5u/Dw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: Renamed Acroform fields and sync the changes to Excel template and codebase
</commit_message>
<xml_diff>
--- a/public/templates/Rekord Template - Grade 4.xlsx
+++ b/public/templates/Rekord Template - Grade 4.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jerwin\Documents\GitHub\rekord\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31092D7-21D8-43C9-9CE7-FAF2008C5B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DAA15D9-658B-46AE-9078-304F5E82997E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="README!" sheetId="5" r:id="rId1"/>
-    <sheet name="Class Info" sheetId="1" r:id="rId2"/>
-    <sheet name="Grades" sheetId="2" r:id="rId3"/>
-    <sheet name="Export" sheetId="3" r:id="rId4"/>
-    <sheet name="data" sheetId="4" r:id="rId5"/>
+    <sheet name="README!" sheetId="6" r:id="rId1"/>
+    <sheet name="Class Info" sheetId="2" r:id="rId2"/>
+    <sheet name="Grades" sheetId="3" r:id="rId3"/>
+    <sheet name="Export" sheetId="4" r:id="rId4"/>
+    <sheet name="data" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" iterate="1" iterateDelta="1E-4"/>
   <extLst>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -84,12 +81,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="137">
   <si>
-    <t>LEARNER'S PERSONAL INFORMATION</t>
-  </si>
-  <si>
-    <t>ELIGIBILITY FOR ELEMENTARY SCHOOL ENROLLMENT</t>
-  </si>
-  <si>
     <t>LRN</t>
   </si>
   <si>
@@ -97,48 +88,6 @@
   </si>
   <si>
     <t>First Name</t>
-  </si>
-  <si>
-    <t>Middle Name</t>
-  </si>
-  <si>
-    <t>Extn.</t>
-  </si>
-  <si>
-    <t>Birthdate (mm/dd/yy)</t>
-  </si>
-  <si>
-    <t>Sex</t>
-  </si>
-  <si>
-    <t>Credential Presented for Grade 1</t>
-  </si>
-  <si>
-    <t>Name of School</t>
-  </si>
-  <si>
-    <t>School Address</t>
-  </si>
-  <si>
-    <t>PEPT Passer Rating</t>
-  </si>
-  <si>
-    <t>Date of Examination</t>
-  </si>
-  <si>
-    <t>Name and Address of Testing Center</t>
-  </si>
-  <si>
-    <t>Other Credentials Presented</t>
-  </si>
-  <si>
-    <t>Remark</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>Kindergarten Certificate of Completion</t>
   </si>
   <si>
     <t>Quarter 1</t>
@@ -195,238 +144,337 @@
     <t>General Average</t>
   </si>
   <si>
+    <t>Rekord</t>
+  </si>
+  <si>
+    <t>This workbook is used to prepare and export student data for Grade 4 SF10-ES generation. Fill in the Class Info and Grades sheets, export the Export sheet as a CSV, and upload it to Rekord to batch-generate ready-to-print PDFs for all your students.</t>
+  </si>
+  <si>
+    <t>Here's a quick guide to get you started with this template:</t>
+  </si>
+  <si>
+    <t>Step 1 — Fill in Class Info</t>
+  </si>
+  <si>
+    <t>Head over to the "Class Info" sheet and start filling in your students' info, one student per row. You can have up to 100 students.</t>
+  </si>
+  <si>
+    <t>Go to Class Info Sheet →</t>
+  </si>
+  <si>
+    <t>Step 2 — Enter Grades</t>
+  </si>
+  <si>
+    <t>Switch to the "Grades" sheet and fill in each student's quarterly grades (Q1–Q4) per subject. Don't worry about the LRN and name columns since those are pulled automatically from Class Info. The Final Rating and General Average are also computed for you, so no need to worry about those.</t>
+  </si>
+  <si>
+    <t>Go to Grades Sheet →</t>
+  </si>
+  <si>
+    <t>Step 3 — Export</t>
+  </si>
+  <si>
+    <t>Go to "Export" sheet (very important), then go to File → Export → Change File Type → CSV (Comma delimited) (*.csv) → Save As. Excel might warn you that only the current sheet will be saved, that's totally fine, just click OK.</t>
+  </si>
+  <si>
+    <t>Go to Export Sheet →</t>
+  </si>
+  <si>
+    <t>Step 4 — Upload to Rekord</t>
+  </si>
+  <si>
+    <t>Go to Rekord, upload the CSV you just saved, fill in the required fields, and hit Process.  In a few seconds, you'll have a ZIP file with a PDF for every student. Donezo! 🎉</t>
+  </si>
+  <si>
+    <t>Go to Rekord →</t>
+  </si>
+  <si>
+    <t>LEARNER'S PERSONAL INFORMATION</t>
+  </si>
+  <si>
+    <t>ELIGIBILITY FOR ELEMENTARY SCHOOL ENROLLMENT</t>
+  </si>
+  <si>
+    <t>Middle Name</t>
+  </si>
+  <si>
+    <t>Extn.</t>
+  </si>
+  <si>
+    <t>Birthdate (mm/dd/yy)</t>
+  </si>
+  <si>
+    <t>Sex</t>
+  </si>
+  <si>
+    <t>Credential Presented for Grade 1</t>
+  </si>
+  <si>
+    <t>Name of School</t>
+  </si>
+  <si>
+    <t>School Address</t>
+  </si>
+  <si>
+    <t>PEPT Passer Rating</t>
+  </si>
+  <si>
+    <t>Date of Examination</t>
+  </si>
+  <si>
+    <t>Name and Address of Testing Center</t>
+  </si>
+  <si>
+    <t>Other Credentials Presented</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
     <t># Read Only</t>
   </si>
   <si>
-    <t>info.lrn</t>
+    <t>learner.lrn</t>
   </si>
   <si>
-    <t>info.last_name</t>
+    <t>learner.last_name</t>
   </si>
   <si>
-    <t>info.first_name</t>
+    <t>learner.first_name</t>
   </si>
   <si>
-    <t>info.middle_name</t>
+    <t>learner.middle_name</t>
   </si>
   <si>
-    <t>info.birthdate</t>
+    <t>learner.extn</t>
   </si>
   <si>
-    <t>info.extn</t>
+    <t>learner.birthdate</t>
   </si>
   <si>
-    <t>info.sex</t>
+    <t>learner.sex</t>
   </si>
   <si>
     <t>credential_presented_for_grade_1</t>
   </si>
   <si>
-    <t>credential.name_of_school</t>
+    <t>enrollment.name_of_school</t>
   </si>
   <si>
-    <t>credential.school_address</t>
+    <t>enrollment.school_address</t>
   </si>
   <si>
-    <t>credential.pept.rating</t>
+    <t>enrollment.pept.rating</t>
   </si>
   <si>
-    <t>credential.pept.date_of_examination</t>
+    <t>enrollment.pept.date_of_examination</t>
   </si>
   <si>
-    <t>credential.pept.name_of_testing_center</t>
+    <t>enrollment.pept.name_of_testing_center</t>
   </si>
   <si>
-    <t>credential.others</t>
+    <t>enrollment.others</t>
   </si>
   <si>
-    <t>scholastic_4.grade.filipino.quarter_1</t>
+    <t>enrollment.remark</t>
   </si>
   <si>
-    <t>scholastic_4.grade.filipino.quarter_2</t>
+    <t>record_4.quarterly.filipino.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.filipino.quarter_3</t>
+    <t>record_4.quarterly.filipino.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.filipino.quarter_4</t>
+    <t>record_4.quarterly.filipino.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.english.quarter_1</t>
+    <t>record_4.quarterly.filipino.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.english.quarter_2</t>
+    <t>record_4.quarterly.english.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.english.quarter_3</t>
+    <t>record_4.quarterly.english.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.english.quarter_4</t>
+    <t>record_4.quarterly.english.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mathematics.quarter_1</t>
+    <t>record_4.quarterly.english.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mathematics.quarter_2</t>
+    <t>record_4.quarterly.mathematics.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mathematics.quarter_3</t>
+    <t>record_4.quarterly.mathematics.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mathematics.quarter_4</t>
+    <t>record_4.quarterly.mathematics.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.science.quarter_1</t>
+    <t>record_4.quarterly.mathematics.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.science.quarter_2</t>
+    <t>record_4.quarterly.science.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.science.quarter_3</t>
+    <t>record_4.quarterly.science.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.science.quarter_4</t>
+    <t>record_4.quarterly.science.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.gmrc.quarter_1</t>
+    <t>record_4.quarterly.science.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.gmrc.quarter_2</t>
+    <t>record_4.quarterly.gmrc.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.gmrc.quarter_3</t>
+    <t>record_4.quarterly.gmrc.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.gmrc.quarter_4</t>
+    <t>record_4.quarterly.gmrc.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.araling_panlipunan.quarter_1</t>
+    <t>record_4.quarterly.gmrc.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.araling_panlipunan.quarter_2</t>
+    <t>record_4.quarterly.araling_panlipunan.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.araling_panlipunan.quarter_3</t>
+    <t>record_4.quarterly.araling_panlipunan.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.araling_panlipunan.quarter_4</t>
+    <t>record_4.quarterly.araling_panlipunan.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.epp.quarter_1</t>
+    <t>record_4.quarterly.araling_panlipunan.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.epp.quarter_2</t>
+    <t>record_4.quarterly.epp.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.epp.quarter_3</t>
+    <t>record_4.quarterly.epp.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.epp.quarter_4</t>
+    <t>record_4.quarterly.epp.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mapeh.quarter_1</t>
+    <t>record_4.quarterly.epp.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mapeh.quarter_2</t>
+    <t>record_4.quarterly.mapeh.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mapeh.quarter_3</t>
+    <t>record_4.quarterly.mapeh.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.mapeh.quarter_4</t>
+    <t>record_4.quarterly.mapeh.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.music_and_arts.quarter_1</t>
+    <t>record_4.quarterly.mapeh.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.music_and_arts.quarter_2</t>
+    <t>record_4.quarterly.music_and_arts.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.music_and_arts.quarter_3</t>
+    <t>record_4.quarterly.music_and_arts.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.music_and_arts.quarter_4</t>
+    <t>record_4.quarterly.music_and_arts.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.physical_education_and_health.quarter_1</t>
+    <t>record_4.quarterly.music_and_arts.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.physical_education_and_health.quarter_2</t>
+    <t>record_4.quarterly.physical_education_and_health.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.physical_education_and_health.quarter_3</t>
+    <t>record_4.quarterly.physical_education_and_health.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.physical_education_and_health.quarter_4</t>
+    <t>record_4.quarterly.physical_education_and_health.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.arabic_language.quarter_1</t>
+    <t>record_4.quarterly.physical_education_and_health.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.arabic_language.quarter_2</t>
+    <t>record_4.quarterly.arabic_language.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.arabic_language.quarter_3</t>
+    <t>record_4.quarterly.arabic_language.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.arabic_language.quarter_4</t>
+    <t>record_4.quarterly.arabic_language.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.grade.islamic_values_education.quarter_1</t>
+    <t>record_4.quarterly.arabic_language.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.grade.islamic_values_education.quarter_2</t>
+    <t>record_4.quarterly.islamic_values_education.quarter_1</t>
   </si>
   <si>
-    <t>scholastic_4.grade.islamic_values_education.quarter_3</t>
+    <t>record_4.quarterly.islamic_values_education.quarter_2</t>
   </si>
   <si>
-    <t>scholastic_4.grade.islamic_values_education.quarter_4</t>
+    <t>record_4.quarterly.islamic_values_education.quarter_3</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.filipino</t>
+    <t>record_4.quarterly.islamic_values_education.quarter_4</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.english</t>
+    <t>record_4.final_rating.filipino</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.mathematics</t>
+    <t>record_4.final_rating.english</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.science</t>
+    <t>record_4.final_rating.mathematics</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.gmrc</t>
+    <t>record_4.final_rating.science</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.araling_panlipunan</t>
+    <t>record_4.final_rating.gmrc</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.epp</t>
+    <t>record_4.final_rating.araling_panlipunan</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.mapeh</t>
+    <t>record_4.final_rating.epp</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.arabic_language</t>
+    <t>record_4.final_rating.mapeh</t>
   </si>
   <si>
-    <t>scholastic_4.final_rating.islamic_values_education</t>
+    <t>record_4.final_rating.arabic_language</t>
   </si>
   <si>
-    <t>scholastic_4.general_average</t>
+    <t>record_4.final_rating.islamic_values_education</t>
+  </si>
+  <si>
+    <t>record_4.general_average</t>
+  </si>
+  <si>
+    <t># Read only</t>
   </si>
   <si>
     <t>sex</t>
   </si>
   <si>
-    <t>Kinder Progress Report</t>
+    <t>M</t>
   </si>
   <si>
     <t>F</t>
   </si>
   <si>
+    <t>Kinder Progress Report</t>
+  </si>
+  <si>
     <t>ECCD Checklist</t>
+  </si>
+  <si>
+    <t>Kindergarten Certificate of Completion</t>
   </si>
   <si>
     <t>Kinder Progress Report, ECCD Checklist</t>
@@ -439,48 +487,6 @@
   </si>
   <si>
     <t>All</t>
-  </si>
-  <si>
-    <t># Read only</t>
-  </si>
-  <si>
-    <t>credential.remark</t>
-  </si>
-  <si>
-    <t>Rekord</t>
-  </si>
-  <si>
-    <t>This workbook is used to prepare and export student data for Grade 4 SF10-ES generation. Fill in the Class Info and Grades sheets, export the Export sheet as a CSV, and upload it to Rekord to batch-generate ready-to-print PDFs for all your students.</t>
-  </si>
-  <si>
-    <t>Step 1 — Fill in Class Info</t>
-  </si>
-  <si>
-    <t>Here's a quick guide to get you started with this template:</t>
-  </si>
-  <si>
-    <t>Switch to the "Grades" sheet and fill in each student's quarterly grades (Q1–Q4) per subject. Don't worry about the LRN and name columns since those are pulled automatically from Class Info. The Final Rating and General Average are also computed for you, so no need to worry about those.</t>
-  </si>
-  <si>
-    <t>Step 2 — Enter Grades</t>
-  </si>
-  <si>
-    <t>Step 3 — Export</t>
-  </si>
-  <si>
-    <t>Go to "Export" sheet (very important), then go to File → Export → Change File Type → CSV (Comma delimited) (*.csv) → Save As. Excel might warn you that only the current sheet will be saved, that's totally fine, just click OK.</t>
-  </si>
-  <si>
-    <t>Step 4 — Upload to Rekord</t>
-  </si>
-  <si>
-    <t>Go to Class Info Sheet →</t>
-  </si>
-  <si>
-    <t>Go to Grades Sheet →</t>
-  </si>
-  <si>
-    <t>Go to Export Sheet →</t>
   </si>
   <si>
     <r>
@@ -505,15 +511,6 @@
       </rPr>
       <t>.</t>
     </r>
-  </si>
-  <si>
-    <t>Head over to the "Class Info" sheet and start filling in your students' info, one student per row. You can have up to 100 students.</t>
-  </si>
-  <si>
-    <t>Go to Rekord →</t>
-  </si>
-  <si>
-    <t>Go to Rekord, upload the CSV you just saved, fill in the required fields, and hit Process.  In a few seconds, you'll have a ZIP file with a PDF for every student. Donezo! 🎉</t>
   </si>
 </sst>
 </file>
@@ -717,7 +714,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -740,12 +737,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -814,6 +848,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -821,10 +858,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -835,32 +878,23 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -868,12 +902,16 @@
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="1" xr:uid="{29B0C132-D4E5-413B-A38D-D4A27A1706DD}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1213,7 +1251,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D9DD6A4-21F3-4506-9045-0B2E3D61FDEB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669AB2C8-AABF-4307-AA9D-9676B5CAE66C}">
   <dimension ref="C1:R19"/>
   <sheetFormatPr defaultRowHeight="15.65" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1223,381 +1261,373 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:18" ht="87.65" customHeight="1" x14ac:dyDescent="1.2">
-      <c r="C1" s="39" t="s">
-        <v>121</v>
-      </c>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
-      <c r="R1" s="39"/>
+      <c r="C1" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
     </row>
     <row r="2" spans="3:18" ht="69.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="38" t="s">
-        <v>122</v>
-      </c>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="38"/>
-      <c r="R2" s="38"/>
+      <c r="C2" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="41"/>
     </row>
     <row r="3" spans="3:18" ht="22.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="40" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
+      <c r="C3" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
+      <c r="I3" s="43"/>
+      <c r="J3" s="43"/>
+      <c r="K3" s="43"/>
+      <c r="L3" s="43"/>
+      <c r="M3" s="43"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43"/>
     </row>
     <row r="4" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="42" t="s">
-        <v>123</v>
-      </c>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="42"/>
-      <c r="L4" s="42"/>
-      <c r="M4" s="42"/>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="42"/>
-      <c r="R4" s="42"/>
+      <c r="C4" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="39"/>
+      <c r="N4" s="39"/>
+      <c r="O4" s="39"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
+      <c r="R4" s="39"/>
     </row>
     <row r="5" spans="3:18" ht="40.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C5" s="41" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-      <c r="O5" s="41"/>
-      <c r="P5" s="41"/>
-      <c r="Q5" s="41"/>
-      <c r="R5" s="41"/>
+      <c r="C5" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
     </row>
     <row r="6" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="37"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="37"/>
-      <c r="O6" s="37"/>
-      <c r="P6" s="37"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="37"/>
+      <c r="C6" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="38"/>
+      <c r="P6" s="38"/>
+      <c r="Q6" s="38"/>
+      <c r="R6" s="38"/>
     </row>
     <row r="7" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42"/>
-      <c r="P7" s="42"/>
-      <c r="Q7" s="42"/>
-      <c r="R7" s="42"/>
+      <c r="C7" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="39"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="39"/>
+      <c r="P7" s="39"/>
+      <c r="Q7" s="39"/>
+      <c r="R7" s="39"/>
     </row>
     <row r="8" spans="3:18" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C8" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="41"/>
-      <c r="P8" s="41"/>
-      <c r="Q8" s="41"/>
-      <c r="R8" s="41"/>
+      <c r="C8" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="37"/>
+      <c r="N8" s="37"/>
+      <c r="O8" s="37"/>
+      <c r="P8" s="37"/>
+      <c r="Q8" s="37"/>
+      <c r="R8" s="37"/>
     </row>
     <row r="9" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="37"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
+      <c r="C9" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
+      <c r="P9" s="38"/>
+      <c r="Q9" s="38"/>
+      <c r="R9" s="38"/>
     </row>
     <row r="10" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C10" s="42" t="s">
-        <v>127</v>
-      </c>
-      <c r="D10" s="42"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="42"/>
-      <c r="L10" s="42"/>
-      <c r="M10" s="42"/>
-      <c r="N10" s="42"/>
-      <c r="O10" s="42"/>
-      <c r="P10" s="42"/>
-      <c r="Q10" s="42"/>
-      <c r="R10" s="42"/>
+      <c r="C10" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
+      <c r="G10" s="39"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="39"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
+      <c r="L10" s="39"/>
+      <c r="M10" s="39"/>
+      <c r="N10" s="39"/>
+      <c r="O10" s="39"/>
+      <c r="P10" s="39"/>
+      <c r="Q10" s="39"/>
+      <c r="R10" s="39"/>
     </row>
     <row r="11" spans="3:18" ht="59.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
-      <c r="N11" s="41"/>
-      <c r="O11" s="41"/>
-      <c r="P11" s="41"/>
-      <c r="Q11" s="41"/>
-      <c r="R11" s="41"/>
+      <c r="C11" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="37"/>
+      <c r="E11" s="37"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="37"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="37"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="37"/>
+      <c r="M11" s="37"/>
+      <c r="N11" s="37"/>
+      <c r="O11" s="37"/>
+      <c r="P11" s="37"/>
+      <c r="Q11" s="37"/>
+      <c r="R11" s="37"/>
     </row>
-    <row r="12" spans="3:18" ht="378.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="43" t="e" vm="1">
+    <row r="12" spans="3:18" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C12" s="40" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="43"/>
-      <c r="Q12" s="43"/>
-      <c r="R12" s="43"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="40"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="40"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="40"/>
     </row>
     <row r="13" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="37"/>
-      <c r="L13" s="37"/>
-      <c r="M13" s="37"/>
-      <c r="N13" s="37"/>
-      <c r="O13" s="37"/>
-      <c r="P13" s="37"/>
-      <c r="Q13" s="37"/>
-      <c r="R13" s="37"/>
+      <c r="C13" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="38"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="38"/>
+      <c r="P13" s="38"/>
+      <c r="Q13" s="38"/>
+      <c r="R13" s="38"/>
     </row>
     <row r="14" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C14" s="42" t="s">
-        <v>129</v>
-      </c>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="42"/>
-      <c r="N14" s="42"/>
-      <c r="O14" s="42"/>
-      <c r="P14" s="42"/>
-      <c r="Q14" s="42"/>
-      <c r="R14" s="42"/>
+      <c r="C14" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
+      <c r="L14" s="39"/>
+      <c r="M14" s="39"/>
+      <c r="N14" s="39"/>
+      <c r="O14" s="39"/>
+      <c r="P14" s="39"/>
+      <c r="Q14" s="39"/>
+      <c r="R14" s="39"/>
     </row>
     <row r="15" spans="3:18" ht="41.35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C15" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="41"/>
-      <c r="K15" s="41"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="41"/>
-      <c r="N15" s="41"/>
-      <c r="O15" s="41"/>
-      <c r="P15" s="41"/>
-      <c r="Q15" s="41"/>
-      <c r="R15" s="41"/>
+      <c r="C15" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="37"/>
+      <c r="E15" s="37"/>
+      <c r="F15" s="37"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="37"/>
+      <c r="J15" s="37"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="37"/>
+      <c r="M15" s="37"/>
+      <c r="N15" s="37"/>
+      <c r="O15" s="37"/>
+      <c r="P15" s="37"/>
+      <c r="Q15" s="37"/>
+      <c r="R15" s="37"/>
     </row>
     <row r="16" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
-      <c r="L16" s="37"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="37"/>
-      <c r="O16" s="37"/>
-      <c r="P16" s="37"/>
-      <c r="Q16" s="37"/>
-      <c r="R16" s="37"/>
+      <c r="C16" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="38"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
+      <c r="N16" s="38"/>
+      <c r="O16" s="38"/>
+      <c r="P16" s="38"/>
+      <c r="Q16" s="38"/>
+      <c r="R16" s="38"/>
     </row>
     <row r="17" spans="3:18" ht="31.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="41" t="s">
-        <v>133</v>
-      </c>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="41"/>
-      <c r="J17" s="41"/>
-      <c r="K17" s="41"/>
-      <c r="L17" s="41"/>
-      <c r="M17" s="41"/>
-      <c r="N17" s="41"/>
-      <c r="O17" s="41"/>
-      <c r="P17" s="41"/>
-      <c r="Q17" s="41"/>
-      <c r="R17" s="41"/>
+      <c r="C17" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="37"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="37"/>
+      <c r="M17" s="37"/>
+      <c r="N17" s="37"/>
+      <c r="O17" s="37"/>
+      <c r="P17" s="37"/>
+      <c r="Q17" s="37"/>
+      <c r="R17" s="37"/>
     </row>
     <row r="18" spans="3:18" ht="63.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="36"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+      <c r="M18" s="34"/>
+      <c r="N18" s="34"/>
+      <c r="O18" s="34"/>
+      <c r="P18" s="34"/>
+      <c r="Q18" s="34"/>
+      <c r="R18" s="34"/>
     </row>
     <row r="19" spans="3:18" ht="30.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="35" t="e" vm="2">
+      <c r="C19" s="36" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="D19" s="34" t="e" vm="3">
+      <c r="D19" s="35" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="C2eitg/wVVV0kyyQJC0VLipqMFRM+3PW1MeezuIv/PreHWXO+QjsttCqX7YqnNPJ2EZxrPDwoJR8DE/zQIjV1w==" saltValue="4eH05uxoVOqJ721VkYCI5w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="17">
-    <mergeCell ref="C17:R17"/>
-    <mergeCell ref="C16:R16"/>
-    <mergeCell ref="C10:R10"/>
-    <mergeCell ref="C11:R11"/>
-    <mergeCell ref="C14:R14"/>
-    <mergeCell ref="C15:R15"/>
-    <mergeCell ref="C12:R12"/>
     <mergeCell ref="C6:R6"/>
     <mergeCell ref="C9:R9"/>
     <mergeCell ref="C13:R13"/>
@@ -1608,21 +1638,29 @@
     <mergeCell ref="C4:R4"/>
     <mergeCell ref="C7:R7"/>
     <mergeCell ref="C8:R8"/>
+    <mergeCell ref="C17:R17"/>
+    <mergeCell ref="C16:R16"/>
+    <mergeCell ref="C10:R10"/>
+    <mergeCell ref="C11:R11"/>
+    <mergeCell ref="C14:R14"/>
+    <mergeCell ref="C15:R15"/>
+    <mergeCell ref="C12:R12"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C6:R6" location="'Class Info'!A1" display="Go to Class Info Sheet →" xr:uid="{8C8433A5-16A5-4B84-8E34-CC7C8D28B64C}"/>
-    <hyperlink ref="C9:R9" location="Grades!A1" display="Go to Grades Sheet →" xr:uid="{37A54A8A-29D1-4B30-9F96-67384A9AB80F}"/>
-    <hyperlink ref="C13:R13" location="Export!A1" display="Go to Export Sheet →" xr:uid="{808C060A-4F33-4C9C-8EAE-ADD7276B5B40}"/>
-    <hyperlink ref="C19" r:id="rId1" display="https://github.com/jrwnnnn/rekord" xr:uid="{340F7352-5064-462C-85BC-12620A945179}"/>
-    <hyperlink ref="C16:R16" r:id="rId2" display="Go to Rekord →" xr:uid="{7BC2C170-D1D1-4303-BB62-FF825A2196EC}"/>
-    <hyperlink ref="D19" r:id="rId3" display="https://github.com/jrwnnnn/rekord/issues/new" xr:uid="{D872846D-0124-4F13-9568-CA87D26DE526}"/>
+    <hyperlink ref="C6:R6" location="'Class Info'!A1" display="Go to Class Info Sheet →" xr:uid="{1C26BCE7-34EA-4843-BC49-47B45D5158D6}"/>
+    <hyperlink ref="C9:R9" location="Grades!A1" display="Go to Grades Sheet →" xr:uid="{B26C73EF-1DD6-4E2A-91CF-C4782032368B}"/>
+    <hyperlink ref="C13:R13" location="Export!A1" display="Go to Export Sheet →" xr:uid="{A25CA826-E450-4159-A32F-DEAC4C6AA570}"/>
+    <hyperlink ref="C19" r:id="rId1" tooltip="View source" display="https://github.com/jrwnnnn/rekord" xr:uid="{7A78B43F-61AE-4709-B1D0-A0E0358D6AB7}"/>
+    <hyperlink ref="C16:R16" r:id="rId2" display="Go to Rekord →" xr:uid="{6766812D-5F8E-4CA1-9BA4-9CBADE087D57}"/>
+    <hyperlink ref="D19" r:id="rId3" tooltip="Report an Issue" display="https://github.com/jrwnnnn/rekord/issues/new" xr:uid="{BA6E77D3-8F0A-44C6-8A8A-61209D05AC39}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O102"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1641,21 +1679,22 @@
     <col min="13" max="13" width="38.5546875" style="16" customWidth="1"/>
     <col min="14" max="14" width="29.88671875" style="16" customWidth="1"/>
     <col min="15" max="15" width="11.44140625" style="16" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="16"/>
+    <col min="16" max="16" width="8.88671875" style="16" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="11" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="11" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="45" t="s">
-        <v>1</v>
+        <v>36</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="47" t="s">
+        <v>37</v>
       </c>
       <c r="I1" s="45"/>
       <c r="J1" s="45"/>
@@ -1663,53 +1702,53 @@
       <c r="L1" s="45"/>
       <c r="M1" s="45"/>
       <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
+      <c r="O1" s="46"/>
     </row>
     <row r="2" spans="1:15" s="11" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>4</v>
-      </c>
       <c r="D2" s="12" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="K2" s="12" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="N2" s="12" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="O2" s="12" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -3413,7 +3452,7 @@
       <c r="O102" s="14"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="wEC5uJWRRXy6psjtSTCRxOe72hcOnC7E6ealfPK+sdUNB5pSced1dAhla01DbY6ByfdHu5aZxEm3qowy6tV0Tg==" saltValue="BrNZpmlhSslY2IKcBmGJcw==" spinCount="100000" sheet="1" formatColumns="0"/>
+  <sheetProtection formatColumns="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="H1:O1"/>
@@ -3423,17 +3462,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{120A8BCC-2D49-40D5-B4EE-8C8C529AE5F2}">
-          <x14:formula1>
-            <xm:f>data!$A$3:$A$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>G3:G102</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7468AB36-F7EB-4AE9-ABCB-FBDD3C61EC3D}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DA79BF08-6B24-4765-9764-C1500A778647}">
           <x14:formula1>
             <xm:f>data!$B$3:$B$10</xm:f>
           </x14:formula1>
           <xm:sqref>H3:H102</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6D0E0026-4147-4E04-AE5B-076C50E1ACB4}">
+          <x14:formula1>
+            <xm:f>data!$A$3:$A$5</xm:f>
+          </x14:formula1>
+          <xm:sqref>G3:G102</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3442,7 +3481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:BL102"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3451,291 +3490,292 @@
     <col min="3" max="3" width="24.5546875" style="1" customWidth="1"/>
     <col min="4" max="10" width="7.77734375" style="18" customWidth="1"/>
     <col min="11" max="12" width="13.88671875" style="18" customWidth="1"/>
-    <col min="13" max="15" width="8.88671875" style="18"/>
-    <col min="16" max="22" width="8.88671875" style="19"/>
+    <col min="13" max="15" width="8.88671875" style="18" customWidth="1"/>
+    <col min="16" max="22" width="8.88671875" style="19" customWidth="1"/>
     <col min="23" max="24" width="13.88671875" style="19" customWidth="1"/>
-    <col min="25" max="27" width="8.88671875" style="19"/>
-    <col min="28" max="34" width="8.88671875" style="20"/>
+    <col min="25" max="27" width="8.88671875" style="19" customWidth="1"/>
+    <col min="28" max="34" width="8.88671875" style="20" customWidth="1"/>
     <col min="35" max="36" width="13.88671875" style="20" customWidth="1"/>
-    <col min="37" max="39" width="8.88671875" style="20"/>
-    <col min="40" max="46" width="8.88671875" style="21"/>
+    <col min="37" max="39" width="8.88671875" style="20" customWidth="1"/>
+    <col min="40" max="46" width="8.88671875" style="21" customWidth="1"/>
     <col min="47" max="48" width="13.88671875" style="21" customWidth="1"/>
-    <col min="49" max="51" width="8.88671875" style="21"/>
-    <col min="52" max="58" width="8.88671875" style="22"/>
+    <col min="49" max="51" width="8.88671875" style="21" customWidth="1"/>
+    <col min="52" max="58" width="8.88671875" style="22" customWidth="1"/>
     <col min="59" max="60" width="13.88671875" style="22" customWidth="1"/>
-    <col min="61" max="63" width="8.88671875" style="22"/>
+    <col min="61" max="63" width="8.88671875" style="22" customWidth="1"/>
     <col min="64" max="64" width="19.77734375" style="22" customWidth="1"/>
-    <col min="65" max="16384" width="8.88671875" style="32"/>
+    <col min="65" max="65" width="8.88671875" style="32" customWidth="1"/>
+    <col min="66" max="16384" width="8.88671875" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" ht="19.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+    <row r="1" spans="1:64" ht="19.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="49" t="s">
+      <c r="D1" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="46"/>
+      <c r="P1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
-      <c r="P1" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="51"/>
-      <c r="Y1" s="51"/>
-      <c r="Z1" s="51"/>
-      <c r="AA1" s="51"/>
-      <c r="AB1" s="46" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC1" s="46"/>
-      <c r="AD1" s="46"/>
-      <c r="AE1" s="46"/>
-      <c r="AF1" s="46"/>
-      <c r="AG1" s="46"/>
-      <c r="AH1" s="46"/>
-      <c r="AI1" s="46"/>
-      <c r="AJ1" s="46"/>
-      <c r="AK1" s="46"/>
-      <c r="AL1" s="46"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="45"/>
+      <c r="AA1" s="46"/>
+      <c r="AB1" s="50" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC1" s="45"/>
+      <c r="AD1" s="45"/>
+      <c r="AE1" s="45"/>
+      <c r="AF1" s="45"/>
+      <c r="AG1" s="45"/>
+      <c r="AH1" s="45"/>
+      <c r="AI1" s="45"/>
+      <c r="AJ1" s="45"/>
+      <c r="AK1" s="45"/>
+      <c r="AL1" s="45"/>
       <c r="AM1" s="46"/>
-      <c r="AN1" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="AO1" s="47"/>
-      <c r="AP1" s="47"/>
-      <c r="AQ1" s="47"/>
-      <c r="AR1" s="47"/>
-      <c r="AS1" s="47"/>
-      <c r="AT1" s="47"/>
-      <c r="AU1" s="47"/>
-      <c r="AV1" s="47"/>
-      <c r="AW1" s="47"/>
-      <c r="AX1" s="47"/>
-      <c r="AY1" s="47"/>
-      <c r="AZ1" s="48" t="s">
-        <v>23</v>
-      </c>
-      <c r="BA1" s="48"/>
-      <c r="BB1" s="48"/>
-      <c r="BC1" s="48"/>
-      <c r="BD1" s="48"/>
-      <c r="BE1" s="48"/>
-      <c r="BF1" s="48"/>
-      <c r="BG1" s="48"/>
-      <c r="BH1" s="48"/>
-      <c r="BI1" s="48"/>
-      <c r="BJ1" s="48"/>
-      <c r="BK1" s="48"/>
-      <c r="BL1" s="48"/>
+      <c r="AN1" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="AO1" s="45"/>
+      <c r="AP1" s="45"/>
+      <c r="AQ1" s="45"/>
+      <c r="AR1" s="45"/>
+      <c r="AS1" s="45"/>
+      <c r="AT1" s="45"/>
+      <c r="AU1" s="45"/>
+      <c r="AV1" s="45"/>
+      <c r="AW1" s="45"/>
+      <c r="AX1" s="45"/>
+      <c r="AY1" s="46"/>
+      <c r="AZ1" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="BA1" s="45"/>
+      <c r="BB1" s="45"/>
+      <c r="BC1" s="45"/>
+      <c r="BD1" s="45"/>
+      <c r="BE1" s="45"/>
+      <c r="BF1" s="45"/>
+      <c r="BG1" s="45"/>
+      <c r="BH1" s="45"/>
+      <c r="BI1" s="45"/>
+      <c r="BJ1" s="45"/>
+      <c r="BK1" s="45"/>
+      <c r="BL1" s="46"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="49"/>
       <c r="B2" s="49"/>
       <c r="C2" s="49"/>
       <c r="D2" s="23" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="K2" s="23" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="L2" s="23" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="M2" s="23" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="N2" s="23" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="O2" s="23" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="P2" s="25" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="Q2" s="25" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="R2" s="25" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="S2" s="25" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="T2" s="25" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="U2" s="25" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="V2" s="25" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="W2" s="25" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="X2" s="25" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="Y2" s="25" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="Z2" s="25" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="AA2" s="25" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="AB2" s="27" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="AC2" s="27" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="AD2" s="27" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="AE2" s="27" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="AF2" s="27" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="AG2" s="27" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="AH2" s="27" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="AI2" s="27" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="AJ2" s="27" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="AK2" s="27" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="AL2" s="27" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="AM2" s="27" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="AN2" s="29" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="AO2" s="29" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="AP2" s="29" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="AQ2" s="29" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="AR2" s="29" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="AS2" s="29" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="AT2" s="29" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="AU2" s="29" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="AV2" s="29" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="AW2" s="29" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="AX2" s="29" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="AY2" s="29" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="AZ2" s="2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="BA2" s="2" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="BB2" s="2" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="BC2" s="2" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="BD2" s="2" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="BE2" s="2" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="BF2" s="2" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="BG2" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="BH2" s="2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="BI2" s="2" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="BJ2" s="2" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="BK2" s="2" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="BL2" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:64" x14ac:dyDescent="0.25">
@@ -3848,7 +3888,7 @@
         <v/>
       </c>
       <c r="BL3" s="5" t="str">
-        <f>IF(COUNT(AZ3:BG3,BJ3:BK3)=0, "", ROUND(AVERAGE(AZ3:BG3,BJ3:BK3), 0))</f>
+        <f t="shared" ref="BL3:BL22" si="12">IF(COUNT(AZ3:BG3,BJ3:BK3)=0, "", ROUND(AVERAGE(AZ3:BG3,BJ3:BK3), 0))</f>
         <v/>
       </c>
     </row>
@@ -3962,7 +4002,7 @@
         <v/>
       </c>
       <c r="BL4" s="5" t="str">
-        <f t="shared" ref="BL4:BL22" si="12">IF(COUNT(AZ4:BG4,BJ4:BK4)=0, "", ROUND(AVERAGE(AZ4:BG4,BJ4:BK4), 0))</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
@@ -13065,17 +13105,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="d5jXvnY3ZYdQOSnLxgdYj536LBKwDTlOueMC+iF9p78qlSXK3Lv+OKGPe0Lr1S7Dix+H/sM2ZVB7ldmziK3NEg==" saltValue="yBTrmWKE0n8/JVmgPP8sZw==" spinCount="100000" sheet="1" formatColumns="0" formatRows="0"/>
   <mergeCells count="8">
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="AB1:AM1"/>
-    <mergeCell ref="AN1:AY1"/>
     <mergeCell ref="AZ1:BL1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:O1"/>
     <mergeCell ref="P1:AA1"/>
+    <mergeCell ref="AN1:AY1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Oops!" error="This cell only accepts whole numbers from 0 to 100. " sqref="D3:AY102" xr:uid="{DBCFBED8-41A7-401D-B236-FC591977D38C}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Oops!" error="This cell only accepts whole numbers from 0 to 100. " sqref="D3:AY102" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
@@ -13086,7 +13126,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:BV102"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
@@ -13098,236 +13138,237 @@
     <col min="7" max="7" width="10.77734375" style="6" customWidth="1"/>
     <col min="8" max="8" width="48.44140625" style="6" customWidth="1"/>
     <col min="9" max="109" width="20.77734375" style="6" customWidth="1"/>
-    <col min="110" max="16384" width="8.88671875" style="6"/>
+    <col min="110" max="110" width="8.88671875" style="6" customWidth="1"/>
+    <col min="111" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:74" s="7" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:74" s="8" customFormat="1" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="O2" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="R2" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="S2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="U2" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="V2" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="W2" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="X2" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="Y2" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="Z2" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="AA2" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB2" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC2" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD2" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE2" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="AF2" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="AG2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="AH2" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="AI2" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="AJ2" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="AK2" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="AL2" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="AM2" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="AN2" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="AO2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AP2" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="AQ2" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="AR2" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="AS2" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="AT2" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="AU2" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="AV2" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="AW2" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="AX2" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="AY2" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="AZ2" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="BA2" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="BB2" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="BC2" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="BD2" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="BE2" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="BF2" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="BG2" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="BH2" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="BI2" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="BJ2" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="BK2" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="BL2" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="BM2" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="BN2" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="BO2" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="BP2" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="BQ2" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="BR2" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="P2" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q2" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="S2" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="X2" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="Z2" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="AA2" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AB2" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="AC2" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="AD2" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="AE2" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF2" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="AG2" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AH2" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI2" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ2" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK2" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="AL2" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AM2" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="AN2" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="AO2" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AP2" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="AQ2" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="AR2" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="AS2" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AT2" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="AU2" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="AV2" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="AW2" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="AX2" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="AY2" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="AZ2" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="BA2" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="BB2" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="BC2" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="BD2" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="BE2" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="BF2" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="BG2" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="BH2" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="BI2" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="BJ2" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="BK2" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="BL2" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="BM2" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="BN2" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="BO2" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="BP2" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="BQ2" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="BR2" s="8" t="s">
-        <v>106</v>
-      </c>
       <c r="BS2" s="8" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="BT2" s="8" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="BU2" s="8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="BV2" s="8" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:74" x14ac:dyDescent="0.3">
@@ -43138,74 +43179,73 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="8.88671875" style="6" customWidth="1"/>
     <col min="2" max="2" width="78.5546875" style="6" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="8.88671875" style="6" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="17" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
-        <v>119</v>
-      </c>
-      <c r="B1" s="52"/>
+      <c r="A1" s="55" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="56"/>
     </row>
     <row r="2" spans="1:2" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>128</v>
+      </c>
       <c r="B5" s="6" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ZGa85aHvu+XZvlJavALoApxoTNydjH58/BGhg3oEikXz34lCtsehB0s02ZDVtLcE+xwXllC5OXo1uRtBOKoUIw==" saltValue="3PKVto87X60xHhO9+IuLBQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="F++1dJ0HTPB+3KMJ5fT0Rjg1YsKYJPuWPT8BH/8sx2PKRRqVaOB1HQq7eKio1/v7mgxTRuuEgdYKCRM6ankuHg==" saltValue="5gWg2Wiju68RPq5L0hPzcw==" spinCount="100000" sheet="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: Updated link to website in excel template
</commit_message>
<xml_diff>
--- a/public/templates/Rekord Template - Grade 4.xlsx
+++ b/public/templates/Rekord Template - Grade 4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jerwin\Documents\GitHub\rekord\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DAA15D9-658B-46AE-9078-304F5E82997E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83C16245-5C9E-4620-AD0C-337FCA059E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -775,11 +775,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -857,17 +858,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -878,13 +878,14 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -909,8 +910,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Hyperlink 2" xfId="1" xr:uid="{29B0C132-D4E5-413B-A38D-D4A27A1706DD}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1261,344 +1266,344 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:18" ht="87.65" customHeight="1" x14ac:dyDescent="1.2">
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
     </row>
     <row r="2" spans="3:18" ht="69.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
-      <c r="R2" s="41"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
     </row>
     <row r="3" spans="3:18" ht="22.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="43" t="s">
+      <c r="C3" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="43"/>
-      <c r="O3" s="43"/>
-      <c r="P3" s="43"/>
-      <c r="Q3" s="43"/>
-      <c r="R3" s="43"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
     </row>
     <row r="4" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="39"/>
-      <c r="O4" s="39"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
-      <c r="R4" s="39"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="46"/>
+      <c r="Q4" s="46"/>
+      <c r="R4" s="46"/>
     </row>
     <row r="5" spans="3:18" ht="40.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="37"/>
-      <c r="M5" s="37"/>
-      <c r="N5" s="37"/>
-      <c r="O5" s="37"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="45"/>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
     </row>
     <row r="6" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="38" t="s">
+      <c r="C6" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="38"/>
-      <c r="Q6" s="38"/>
-      <c r="R6" s="38"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="41"/>
+      <c r="L6" s="41"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
     </row>
     <row r="7" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39"/>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="39"/>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-      <c r="R7" s="39"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="46"/>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
+      <c r="O7" s="46"/>
+      <c r="P7" s="46"/>
+      <c r="Q7" s="46"/>
+      <c r="R7" s="46"/>
     </row>
     <row r="8" spans="3:18" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="37"/>
-      <c r="M8" s="37"/>
-      <c r="N8" s="37"/>
-      <c r="O8" s="37"/>
-      <c r="P8" s="37"/>
-      <c r="Q8" s="37"/>
-      <c r="R8" s="37"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+      <c r="L8" s="45"/>
+      <c r="M8" s="45"/>
+      <c r="N8" s="45"/>
+      <c r="O8" s="45"/>
+      <c r="P8" s="45"/>
+      <c r="Q8" s="45"/>
+      <c r="R8" s="45"/>
     </row>
     <row r="9" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
-      <c r="O9" s="38"/>
-      <c r="P9" s="38"/>
-      <c r="Q9" s="38"/>
-      <c r="R9" s="38"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41"/>
+      <c r="L9" s="41"/>
+      <c r="M9" s="41"/>
+      <c r="N9" s="41"/>
+      <c r="O9" s="41"/>
+      <c r="P9" s="41"/>
+      <c r="Q9" s="41"/>
+      <c r="R9" s="41"/>
     </row>
     <row r="10" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="39"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="46"/>
+      <c r="K10" s="46"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46"/>
+      <c r="P10" s="46"/>
+      <c r="Q10" s="46"/>
+      <c r="R10" s="46"/>
     </row>
     <row r="11" spans="3:18" ht="59.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="37" t="s">
+      <c r="C11" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="37"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
-      <c r="L11" s="37"/>
-      <c r="M11" s="37"/>
-      <c r="N11" s="37"/>
-      <c r="O11" s="37"/>
-      <c r="P11" s="37"/>
-      <c r="Q11" s="37"/>
-      <c r="R11" s="37"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
     </row>
     <row r="12" spans="3:18" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="40" t="e" vm="1">
+      <c r="C12" s="47" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="40"/>
-      <c r="P12" s="40"/>
-      <c r="Q12" s="40"/>
-      <c r="R12" s="40"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="47"/>
+      <c r="J12" s="47"/>
+      <c r="K12" s="47"/>
+      <c r="L12" s="47"/>
+      <c r="M12" s="47"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="47"/>
+      <c r="P12" s="47"/>
+      <c r="Q12" s="47"/>
+      <c r="R12" s="47"/>
     </row>
     <row r="13" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="38"/>
-      <c r="K13" s="38"/>
-      <c r="L13" s="38"/>
-      <c r="M13" s="38"/>
-      <c r="N13" s="38"/>
-      <c r="O13" s="38"/>
-      <c r="P13" s="38"/>
-      <c r="Q13" s="38"/>
-      <c r="R13" s="38"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="41"/>
+      <c r="I13" s="41"/>
+      <c r="J13" s="41"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="41"/>
+      <c r="M13" s="41"/>
+      <c r="N13" s="41"/>
+      <c r="O13" s="41"/>
+      <c r="P13" s="41"/>
+      <c r="Q13" s="41"/>
+      <c r="R13" s="41"/>
     </row>
     <row r="14" spans="3:18" ht="23.8" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
-      <c r="H14" s="39"/>
-      <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
-      <c r="K14" s="39"/>
-      <c r="L14" s="39"/>
-      <c r="M14" s="39"/>
-      <c r="N14" s="39"/>
-      <c r="O14" s="39"/>
-      <c r="P14" s="39"/>
-      <c r="Q14" s="39"/>
-      <c r="R14" s="39"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="46"/>
+      <c r="K14" s="46"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="46"/>
+      <c r="Q14" s="46"/>
+      <c r="R14" s="46"/>
     </row>
     <row r="15" spans="3:18" ht="41.35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C15" s="37" t="s">
+      <c r="C15" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="37"/>
-      <c r="K15" s="37"/>
-      <c r="L15" s="37"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="37"/>
-      <c r="O15" s="37"/>
-      <c r="P15" s="37"/>
-      <c r="Q15" s="37"/>
-      <c r="R15" s="37"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="45"/>
+      <c r="R15" s="45"/>
     </row>
     <row r="16" spans="3:18" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="38"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="38"/>
-      <c r="N16" s="38"/>
-      <c r="O16" s="38"/>
-      <c r="P16" s="38"/>
-      <c r="Q16" s="38"/>
-      <c r="R16" s="38"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="57"/>
+      <c r="K16" s="57"/>
+      <c r="L16" s="57"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="57"/>
+      <c r="O16" s="57"/>
+      <c r="P16" s="57"/>
+      <c r="Q16" s="57"/>
+      <c r="R16" s="57"/>
     </row>
     <row r="17" spans="3:18" ht="31.95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="37" t="s">
+      <c r="C17" s="45" t="s">
         <v>136</v>
       </c>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="37"/>
-      <c r="K17" s="37"/>
-      <c r="L17" s="37"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="37"/>
-      <c r="O17" s="37"/>
-      <c r="P17" s="37"/>
-      <c r="Q17" s="37"/>
-      <c r="R17" s="37"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
+      <c r="O17" s="45"/>
+      <c r="P17" s="45"/>
+      <c r="Q17" s="45"/>
+      <c r="R17" s="45"/>
     </row>
     <row r="18" spans="3:18" ht="63.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="34"/>
@@ -1627,7 +1632,15 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="SdYvLbnJMuV1DOKqXJJ7VqrXjL2BaydhpmJ4FWVsO19ICFK8Pv06D5QwOpwoeF8g0Qdqp0IkTR+ZdxM6AZlvmg==" saltValue="gjnaCvFyidHxtRMd4alamg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="17">
+    <mergeCell ref="C17:R17"/>
+    <mergeCell ref="C16:R16"/>
+    <mergeCell ref="C10:R10"/>
+    <mergeCell ref="C11:R11"/>
+    <mergeCell ref="C14:R14"/>
+    <mergeCell ref="C15:R15"/>
+    <mergeCell ref="C12:R12"/>
     <mergeCell ref="C6:R6"/>
     <mergeCell ref="C9:R9"/>
     <mergeCell ref="C13:R13"/>
@@ -1638,13 +1651,6 @@
     <mergeCell ref="C4:R4"/>
     <mergeCell ref="C7:R7"/>
     <mergeCell ref="C8:R8"/>
-    <mergeCell ref="C17:R17"/>
-    <mergeCell ref="C16:R16"/>
-    <mergeCell ref="C10:R10"/>
-    <mergeCell ref="C11:R11"/>
-    <mergeCell ref="C14:R14"/>
-    <mergeCell ref="C15:R15"/>
-    <mergeCell ref="C12:R12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C6:R6" location="'Class Info'!A1" display="Go to Class Info Sheet →" xr:uid="{1C26BCE7-34EA-4843-BC49-47B45D5158D6}"/>
@@ -1684,25 +1690,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="11" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="47" t="s">
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="46"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="39"/>
     </row>
     <row r="2" spans="1:15" s="11" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -3452,7 +3458,7 @@
       <c r="O102" s="14"/>
     </row>
   </sheetData>
-  <sheetProtection formatColumns="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="rO0FymHWrm2cndVihXGa09SLIFKnOaVQdVSn4BfwnK3pEo+FVKOeyMsTrc3BMC9Cu0CBOgD1Yrppz0X1y0Ng9w==" saltValue="RqfP+AcVfH2BzTQnsPHm9w==" spinCount="100000" sheet="1" formatColumns="0"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="H1:O1"/>
@@ -3521,74 +3527,74 @@
       <c r="D1" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="46"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="39"/>
       <c r="P1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
-      <c r="X1" s="45"/>
-      <c r="Y1" s="45"/>
-      <c r="Z1" s="45"/>
-      <c r="AA1" s="46"/>
+      <c r="Q1" s="38"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="38"/>
+      <c r="U1" s="38"/>
+      <c r="V1" s="38"/>
+      <c r="W1" s="38"/>
+      <c r="X1" s="38"/>
+      <c r="Y1" s="38"/>
+      <c r="Z1" s="38"/>
+      <c r="AA1" s="39"/>
       <c r="AB1" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AC1" s="45"/>
-      <c r="AD1" s="45"/>
-      <c r="AE1" s="45"/>
-      <c r="AF1" s="45"/>
-      <c r="AG1" s="45"/>
-      <c r="AH1" s="45"/>
-      <c r="AI1" s="45"/>
-      <c r="AJ1" s="45"/>
-      <c r="AK1" s="45"/>
-      <c r="AL1" s="45"/>
-      <c r="AM1" s="46"/>
+      <c r="AC1" s="38"/>
+      <c r="AD1" s="38"/>
+      <c r="AE1" s="38"/>
+      <c r="AF1" s="38"/>
+      <c r="AG1" s="38"/>
+      <c r="AH1" s="38"/>
+      <c r="AI1" s="38"/>
+      <c r="AJ1" s="38"/>
+      <c r="AK1" s="38"/>
+      <c r="AL1" s="38"/>
+      <c r="AM1" s="39"/>
       <c r="AN1" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="AO1" s="45"/>
-      <c r="AP1" s="45"/>
-      <c r="AQ1" s="45"/>
-      <c r="AR1" s="45"/>
-      <c r="AS1" s="45"/>
-      <c r="AT1" s="45"/>
-      <c r="AU1" s="45"/>
-      <c r="AV1" s="45"/>
-      <c r="AW1" s="45"/>
-      <c r="AX1" s="45"/>
-      <c r="AY1" s="46"/>
+      <c r="AO1" s="38"/>
+      <c r="AP1" s="38"/>
+      <c r="AQ1" s="38"/>
+      <c r="AR1" s="38"/>
+      <c r="AS1" s="38"/>
+      <c r="AT1" s="38"/>
+      <c r="AU1" s="38"/>
+      <c r="AV1" s="38"/>
+      <c r="AW1" s="38"/>
+      <c r="AX1" s="38"/>
+      <c r="AY1" s="39"/>
       <c r="AZ1" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="BA1" s="45"/>
-      <c r="BB1" s="45"/>
-      <c r="BC1" s="45"/>
-      <c r="BD1" s="45"/>
-      <c r="BE1" s="45"/>
-      <c r="BF1" s="45"/>
-      <c r="BG1" s="45"/>
-      <c r="BH1" s="45"/>
-      <c r="BI1" s="45"/>
-      <c r="BJ1" s="45"/>
-      <c r="BK1" s="45"/>
-      <c r="BL1" s="46"/>
+      <c r="BA1" s="38"/>
+      <c r="BB1" s="38"/>
+      <c r="BC1" s="38"/>
+      <c r="BD1" s="38"/>
+      <c r="BE1" s="38"/>
+      <c r="BF1" s="38"/>
+      <c r="BG1" s="38"/>
+      <c r="BH1" s="38"/>
+      <c r="BI1" s="38"/>
+      <c r="BJ1" s="38"/>
+      <c r="BK1" s="38"/>
+      <c r="BL1" s="39"/>
     </row>
     <row r="2" spans="1:64" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="49"/>

</xml_diff>